<commit_message>
Fill Task 2 with Appendix 1 data; split Anton's workbook into two sheets
Anton: column 14 (profit from sales), Maksim: column 2 (headcount).
Word and Excel versions for both students now contain the full solution.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JfCGfJiRYnzaYCvcSFBTpx
</commit_message>
<xml_diff>
--- a/Статистика_Вариант_1/Вершков_Максим_Вариант_1.xlsx
+++ b/Статистика_Вариант_1/Вершков_Максим_Вариант_1.xlsx
@@ -57,7 +57,7 @@
     <t xml:space="preserve">Выборка по возрастанию:</t>
   </si>
   <si>
-    <t xml:space="preserve">Фамилия на В - колонка 2 табл. 1 приложения 1</t>
+    <t xml:space="preserve">Фамилия на В - колонка 2 табл. 1 приложения 1 (численность ППП, чел.)</t>
   </si>
   <si>
     <t xml:space="preserve">Из 10 предприятий задачи 1 случайно без повторения выбираем 3</t>
@@ -1097,19 +1097,39 @@
       <c r="A7" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="B7" s="2"/>
-      <c r="C7" s="2"/>
-      <c r="D7" s="2"/>
-      <c r="E7" s="2"/>
-      <c r="F7" s="2"/>
-      <c r="G7" s="2"/>
-      <c r="H7" s="2"/>
-      <c r="I7" s="2"/>
-      <c r="J7" s="2"/>
-      <c r="K7" s="2"/>
+      <c r="B7" s="2" t="n">
+        <v>253</v>
+      </c>
+      <c r="C7" s="2" t="n">
+        <v>447</v>
+      </c>
+      <c r="D7" s="2" t="n">
+        <v>669</v>
+      </c>
+      <c r="E7" s="2" t="n">
+        <v>278</v>
+      </c>
+      <c r="F7" s="2" t="n">
+        <v>53</v>
+      </c>
+      <c r="G7" s="2" t="n">
+        <v>260</v>
+      </c>
+      <c r="H7" s="2" t="n">
+        <v>250</v>
+      </c>
+      <c r="I7" s="2" t="n">
+        <v>305</v>
+      </c>
+      <c r="J7" s="2" t="n">
+        <v>162</v>
+      </c>
+      <c r="K7" s="2" t="n">
+        <v>637</v>
+      </c>
       <c r="L7" s="2" t="n">
         <f aca="false">SUM(B7:K7)</f>
-        <v>0</v>
+        <v>3314</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1123,7 +1143,7 @@
       </c>
       <c r="D10" s="4" t="n">
         <f aca="false">L7/10</f>
-        <v>0</v>
+        <v>331.4</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1167,7 +1187,7 @@
       </c>
       <c r="E14" s="2" t="n">
         <f aca="false">INDEX($B$7:$K$7,C14)</f>
-        <v>0</v>
+        <v>250</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1189,7 +1209,7 @@
       </c>
       <c r="E15" s="2" t="n">
         <f aca="false">INDEX($B$7:$K$7,C15)</f>
-        <v>0</v>
+        <v>305</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1211,7 +1231,7 @@
       </c>
       <c r="E16" s="2" t="n">
         <f aca="false">INDEX($B$7:$K$7,C16)</f>
-        <v>0</v>
+        <v>637</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1220,7 +1240,7 @@
       </c>
       <c r="D18" s="4" t="n">
         <f aca="false">SUM(E14:E16)/3</f>
-        <v>0</v>
+        <v>397.333333333333</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1229,7 +1249,7 @@
       </c>
       <c r="D19" s="4" t="n">
         <f aca="false">D18-D10</f>
-        <v>0</v>
+        <v>65.9333333333333</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1243,7 +1263,7 @@
       </c>
       <c r="D22" s="4" t="n">
         <f aca="false">AVERAGE(Выборки!F2:F121)</f>
-        <v>0</v>
+        <v>331.4</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1252,13 +1272,13 @@
       </c>
       <c r="D23" s="4" t="n">
         <f aca="false">D10</f>
-        <v>0</v>
+        <v>331.4</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="1" t="str">
         <f aca="false">IF(COUNT(B7:K7)&lt;10,"впиши значения x из приложения 1",IF(ABS(D22-D23)&lt;0.000001,"Совпадает, значит выборочная средняя несмещенная","Не совпадает"))</f>
-        <v>впиши значения x из приложения 1</v>
+        <v>Совпадает, значит выборочная средняя несмещенная</v>
       </c>
     </row>
   </sheetData>
@@ -1307,7 +1327,7 @@
       </c>
       <c r="I1" s="4" t="n">
         <f aca="false">MIN(F2:F121)</f>
-        <v>0</v>
+        <v>155</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1320,26 +1340,26 @@
       </c>
       <c r="C2" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,1)</f>
-        <v>0</v>
+        <v>253</v>
       </c>
       <c r="D2" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,2)</f>
-        <v>0</v>
+        <v>447</v>
       </c>
       <c r="E2" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,3)</f>
-        <v>0</v>
+        <v>669</v>
       </c>
       <c r="F2" s="5" t="n">
         <f aca="false">(C2+D2+E2)/3</f>
-        <v>0</v>
+        <v>456.333333333333</v>
       </c>
       <c r="H2" s="1" t="s">
         <v>34</v>
       </c>
       <c r="I2" s="4" t="n">
         <f aca="false">MAX(F2:F121)</f>
-        <v>0</v>
+        <v>584.333333333333</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1352,19 +1372,19 @@
       </c>
       <c r="C3" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,1)</f>
-        <v>0</v>
+        <v>253</v>
       </c>
       <c r="D3" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,2)</f>
-        <v>0</v>
+        <v>447</v>
       </c>
       <c r="E3" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,4)</f>
-        <v>0</v>
+        <v>278</v>
       </c>
       <c r="F3" s="5" t="n">
         <f aca="false">(C3+D3+E3)/3</f>
-        <v>0</v>
+        <v>326</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1377,19 +1397,19 @@
       </c>
       <c r="C4" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,1)</f>
-        <v>0</v>
+        <v>253</v>
       </c>
       <c r="D4" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,2)</f>
-        <v>0</v>
+        <v>447</v>
       </c>
       <c r="E4" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,5)</f>
-        <v>0</v>
+        <v>53</v>
       </c>
       <c r="F4" s="5" t="n">
         <f aca="false">(C4+D4+E4)/3</f>
-        <v>0</v>
+        <v>251</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1402,19 +1422,19 @@
       </c>
       <c r="C5" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,1)</f>
-        <v>0</v>
+        <v>253</v>
       </c>
       <c r="D5" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,2)</f>
-        <v>0</v>
+        <v>447</v>
       </c>
       <c r="E5" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,6)</f>
-        <v>0</v>
+        <v>260</v>
       </c>
       <c r="F5" s="5" t="n">
         <f aca="false">(C5+D5+E5)/3</f>
-        <v>0</v>
+        <v>320</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1427,19 +1447,19 @@
       </c>
       <c r="C6" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,1)</f>
-        <v>0</v>
+        <v>253</v>
       </c>
       <c r="D6" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,2)</f>
-        <v>0</v>
+        <v>447</v>
       </c>
       <c r="E6" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,7)</f>
-        <v>0</v>
+        <v>250</v>
       </c>
       <c r="F6" s="5" t="n">
         <f aca="false">(C6+D6+E6)/3</f>
-        <v>0</v>
+        <v>316.666666666667</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1452,19 +1472,19 @@
       </c>
       <c r="C7" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,1)</f>
-        <v>0</v>
+        <v>253</v>
       </c>
       <c r="D7" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,2)</f>
-        <v>0</v>
+        <v>447</v>
       </c>
       <c r="E7" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,8)</f>
-        <v>0</v>
+        <v>305</v>
       </c>
       <c r="F7" s="5" t="n">
         <f aca="false">(C7+D7+E7)/3</f>
-        <v>0</v>
+        <v>335</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1477,19 +1497,19 @@
       </c>
       <c r="C8" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,1)</f>
-        <v>0</v>
+        <v>253</v>
       </c>
       <c r="D8" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,2)</f>
-        <v>0</v>
+        <v>447</v>
       </c>
       <c r="E8" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,9)</f>
-        <v>0</v>
+        <v>162</v>
       </c>
       <c r="F8" s="5" t="n">
         <f aca="false">(C8+D8+E8)/3</f>
-        <v>0</v>
+        <v>287.333333333333</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1502,19 +1522,19 @@
       </c>
       <c r="C9" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,1)</f>
-        <v>0</v>
+        <v>253</v>
       </c>
       <c r="D9" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,2)</f>
-        <v>0</v>
+        <v>447</v>
       </c>
       <c r="E9" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,10)</f>
-        <v>0</v>
+        <v>637</v>
       </c>
       <c r="F9" s="5" t="n">
         <f aca="false">(C9+D9+E9)/3</f>
-        <v>0</v>
+        <v>445.666666666667</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1527,19 +1547,19 @@
       </c>
       <c r="C10" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,1)</f>
-        <v>0</v>
+        <v>253</v>
       </c>
       <c r="D10" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,3)</f>
-        <v>0</v>
+        <v>669</v>
       </c>
       <c r="E10" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,4)</f>
-        <v>0</v>
+        <v>278</v>
       </c>
       <c r="F10" s="5" t="n">
         <f aca="false">(C10+D10+E10)/3</f>
-        <v>0</v>
+        <v>400</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1552,19 +1572,19 @@
       </c>
       <c r="C11" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,1)</f>
-        <v>0</v>
+        <v>253</v>
       </c>
       <c r="D11" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,3)</f>
-        <v>0</v>
+        <v>669</v>
       </c>
       <c r="E11" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,5)</f>
-        <v>0</v>
+        <v>53</v>
       </c>
       <c r="F11" s="5" t="n">
         <f aca="false">(C11+D11+E11)/3</f>
-        <v>0</v>
+        <v>325</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1577,19 +1597,19 @@
       </c>
       <c r="C12" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,1)</f>
-        <v>0</v>
+        <v>253</v>
       </c>
       <c r="D12" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,3)</f>
-        <v>0</v>
+        <v>669</v>
       </c>
       <c r="E12" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,6)</f>
-        <v>0</v>
+        <v>260</v>
       </c>
       <c r="F12" s="5" t="n">
         <f aca="false">(C12+D12+E12)/3</f>
-        <v>0</v>
+        <v>394</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1602,19 +1622,19 @@
       </c>
       <c r="C13" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,1)</f>
-        <v>0</v>
+        <v>253</v>
       </c>
       <c r="D13" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,3)</f>
-        <v>0</v>
+        <v>669</v>
       </c>
       <c r="E13" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,7)</f>
-        <v>0</v>
+        <v>250</v>
       </c>
       <c r="F13" s="5" t="n">
         <f aca="false">(C13+D13+E13)/3</f>
-        <v>0</v>
+        <v>390.666666666667</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1627,19 +1647,19 @@
       </c>
       <c r="C14" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,1)</f>
-        <v>0</v>
+        <v>253</v>
       </c>
       <c r="D14" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,3)</f>
-        <v>0</v>
+        <v>669</v>
       </c>
       <c r="E14" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,8)</f>
-        <v>0</v>
+        <v>305</v>
       </c>
       <c r="F14" s="5" t="n">
         <f aca="false">(C14+D14+E14)/3</f>
-        <v>0</v>
+        <v>409</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1652,19 +1672,19 @@
       </c>
       <c r="C15" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,1)</f>
-        <v>0</v>
+        <v>253</v>
       </c>
       <c r="D15" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,3)</f>
-        <v>0</v>
+        <v>669</v>
       </c>
       <c r="E15" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,9)</f>
-        <v>0</v>
+        <v>162</v>
       </c>
       <c r="F15" s="5" t="n">
         <f aca="false">(C15+D15+E15)/3</f>
-        <v>0</v>
+        <v>361.333333333333</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1677,19 +1697,19 @@
       </c>
       <c r="C16" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,1)</f>
-        <v>0</v>
+        <v>253</v>
       </c>
       <c r="D16" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,3)</f>
-        <v>0</v>
+        <v>669</v>
       </c>
       <c r="E16" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,10)</f>
-        <v>0</v>
+        <v>637</v>
       </c>
       <c r="F16" s="5" t="n">
         <f aca="false">(C16+D16+E16)/3</f>
-        <v>0</v>
+        <v>519.666666666667</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1702,19 +1722,19 @@
       </c>
       <c r="C17" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,1)</f>
-        <v>0</v>
+        <v>253</v>
       </c>
       <c r="D17" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,4)</f>
-        <v>0</v>
+        <v>278</v>
       </c>
       <c r="E17" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,5)</f>
-        <v>0</v>
+        <v>53</v>
       </c>
       <c r="F17" s="5" t="n">
         <f aca="false">(C17+D17+E17)/3</f>
-        <v>0</v>
+        <v>194.666666666667</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1727,19 +1747,19 @@
       </c>
       <c r="C18" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,1)</f>
-        <v>0</v>
+        <v>253</v>
       </c>
       <c r="D18" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,4)</f>
-        <v>0</v>
+        <v>278</v>
       </c>
       <c r="E18" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,6)</f>
-        <v>0</v>
+        <v>260</v>
       </c>
       <c r="F18" s="5" t="n">
         <f aca="false">(C18+D18+E18)/3</f>
-        <v>0</v>
+        <v>263.666666666667</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1752,19 +1772,19 @@
       </c>
       <c r="C19" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,1)</f>
-        <v>0</v>
+        <v>253</v>
       </c>
       <c r="D19" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,4)</f>
-        <v>0</v>
+        <v>278</v>
       </c>
       <c r="E19" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,7)</f>
-        <v>0</v>
+        <v>250</v>
       </c>
       <c r="F19" s="5" t="n">
         <f aca="false">(C19+D19+E19)/3</f>
-        <v>0</v>
+        <v>260.333333333333</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1777,19 +1797,19 @@
       </c>
       <c r="C20" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,1)</f>
-        <v>0</v>
+        <v>253</v>
       </c>
       <c r="D20" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,4)</f>
-        <v>0</v>
+        <v>278</v>
       </c>
       <c r="E20" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,8)</f>
-        <v>0</v>
+        <v>305</v>
       </c>
       <c r="F20" s="5" t="n">
         <f aca="false">(C20+D20+E20)/3</f>
-        <v>0</v>
+        <v>278.666666666667</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1802,19 +1822,19 @@
       </c>
       <c r="C21" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,1)</f>
-        <v>0</v>
+        <v>253</v>
       </c>
       <c r="D21" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,4)</f>
-        <v>0</v>
+        <v>278</v>
       </c>
       <c r="E21" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,9)</f>
-        <v>0</v>
+        <v>162</v>
       </c>
       <c r="F21" s="5" t="n">
         <f aca="false">(C21+D21+E21)/3</f>
-        <v>0</v>
+        <v>231</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1827,19 +1847,19 @@
       </c>
       <c r="C22" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,1)</f>
-        <v>0</v>
+        <v>253</v>
       </c>
       <c r="D22" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,4)</f>
-        <v>0</v>
+        <v>278</v>
       </c>
       <c r="E22" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,10)</f>
-        <v>0</v>
+        <v>637</v>
       </c>
       <c r="F22" s="5" t="n">
         <f aca="false">(C22+D22+E22)/3</f>
-        <v>0</v>
+        <v>389.333333333333</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1852,19 +1872,19 @@
       </c>
       <c r="C23" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,1)</f>
-        <v>0</v>
+        <v>253</v>
       </c>
       <c r="D23" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,5)</f>
-        <v>0</v>
+        <v>53</v>
       </c>
       <c r="E23" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,6)</f>
-        <v>0</v>
+        <v>260</v>
       </c>
       <c r="F23" s="5" t="n">
         <f aca="false">(C23+D23+E23)/3</f>
-        <v>0</v>
+        <v>188.666666666667</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1877,19 +1897,19 @@
       </c>
       <c r="C24" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,1)</f>
-        <v>0</v>
+        <v>253</v>
       </c>
       <c r="D24" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,5)</f>
-        <v>0</v>
+        <v>53</v>
       </c>
       <c r="E24" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,7)</f>
-        <v>0</v>
+        <v>250</v>
       </c>
       <c r="F24" s="5" t="n">
         <f aca="false">(C24+D24+E24)/3</f>
-        <v>0</v>
+        <v>185.333333333333</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1902,19 +1922,19 @@
       </c>
       <c r="C25" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,1)</f>
-        <v>0</v>
+        <v>253</v>
       </c>
       <c r="D25" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,5)</f>
-        <v>0</v>
+        <v>53</v>
       </c>
       <c r="E25" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,8)</f>
-        <v>0</v>
+        <v>305</v>
       </c>
       <c r="F25" s="5" t="n">
         <f aca="false">(C25+D25+E25)/3</f>
-        <v>0</v>
+        <v>203.666666666667</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1927,19 +1947,19 @@
       </c>
       <c r="C26" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,1)</f>
-        <v>0</v>
+        <v>253</v>
       </c>
       <c r="D26" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,5)</f>
-        <v>0</v>
+        <v>53</v>
       </c>
       <c r="E26" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,9)</f>
-        <v>0</v>
+        <v>162</v>
       </c>
       <c r="F26" s="5" t="n">
         <f aca="false">(C26+D26+E26)/3</f>
-        <v>0</v>
+        <v>156</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1952,19 +1972,19 @@
       </c>
       <c r="C27" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,1)</f>
-        <v>0</v>
+        <v>253</v>
       </c>
       <c r="D27" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,5)</f>
-        <v>0</v>
+        <v>53</v>
       </c>
       <c r="E27" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,10)</f>
-        <v>0</v>
+        <v>637</v>
       </c>
       <c r="F27" s="5" t="n">
         <f aca="false">(C27+D27+E27)/3</f>
-        <v>0</v>
+        <v>314.333333333333</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1977,19 +1997,19 @@
       </c>
       <c r="C28" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,1)</f>
-        <v>0</v>
+        <v>253</v>
       </c>
       <c r="D28" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,6)</f>
-        <v>0</v>
+        <v>260</v>
       </c>
       <c r="E28" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,7)</f>
-        <v>0</v>
+        <v>250</v>
       </c>
       <c r="F28" s="5" t="n">
         <f aca="false">(C28+D28+E28)/3</f>
-        <v>0</v>
+        <v>254.333333333333</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2002,19 +2022,19 @@
       </c>
       <c r="C29" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,1)</f>
-        <v>0</v>
+        <v>253</v>
       </c>
       <c r="D29" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,6)</f>
-        <v>0</v>
+        <v>260</v>
       </c>
       <c r="E29" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,8)</f>
-        <v>0</v>
+        <v>305</v>
       </c>
       <c r="F29" s="5" t="n">
         <f aca="false">(C29+D29+E29)/3</f>
-        <v>0</v>
+        <v>272.666666666667</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2027,19 +2047,19 @@
       </c>
       <c r="C30" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,1)</f>
-        <v>0</v>
+        <v>253</v>
       </c>
       <c r="D30" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,6)</f>
-        <v>0</v>
+        <v>260</v>
       </c>
       <c r="E30" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,9)</f>
-        <v>0</v>
+        <v>162</v>
       </c>
       <c r="F30" s="5" t="n">
         <f aca="false">(C30+D30+E30)/3</f>
-        <v>0</v>
+        <v>225</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2052,19 +2072,19 @@
       </c>
       <c r="C31" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,1)</f>
-        <v>0</v>
+        <v>253</v>
       </c>
       <c r="D31" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,6)</f>
-        <v>0</v>
+        <v>260</v>
       </c>
       <c r="E31" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,10)</f>
-        <v>0</v>
+        <v>637</v>
       </c>
       <c r="F31" s="5" t="n">
         <f aca="false">(C31+D31+E31)/3</f>
-        <v>0</v>
+        <v>383.333333333333</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2077,19 +2097,19 @@
       </c>
       <c r="C32" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,1)</f>
-        <v>0</v>
+        <v>253</v>
       </c>
       <c r="D32" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,7)</f>
-        <v>0</v>
+        <v>250</v>
       </c>
       <c r="E32" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,8)</f>
-        <v>0</v>
+        <v>305</v>
       </c>
       <c r="F32" s="5" t="n">
         <f aca="false">(C32+D32+E32)/3</f>
-        <v>0</v>
+        <v>269.333333333333</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2102,19 +2122,19 @@
       </c>
       <c r="C33" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,1)</f>
-        <v>0</v>
+        <v>253</v>
       </c>
       <c r="D33" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,7)</f>
-        <v>0</v>
+        <v>250</v>
       </c>
       <c r="E33" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,9)</f>
-        <v>0</v>
+        <v>162</v>
       </c>
       <c r="F33" s="5" t="n">
         <f aca="false">(C33+D33+E33)/3</f>
-        <v>0</v>
+        <v>221.666666666667</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2127,19 +2147,19 @@
       </c>
       <c r="C34" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,1)</f>
-        <v>0</v>
+        <v>253</v>
       </c>
       <c r="D34" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,7)</f>
-        <v>0</v>
+        <v>250</v>
       </c>
       <c r="E34" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,10)</f>
-        <v>0</v>
+        <v>637</v>
       </c>
       <c r="F34" s="5" t="n">
         <f aca="false">(C34+D34+E34)/3</f>
-        <v>0</v>
+        <v>380</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2152,19 +2172,19 @@
       </c>
       <c r="C35" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,1)</f>
-        <v>0</v>
+        <v>253</v>
       </c>
       <c r="D35" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,8)</f>
-        <v>0</v>
+        <v>305</v>
       </c>
       <c r="E35" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,9)</f>
-        <v>0</v>
+        <v>162</v>
       </c>
       <c r="F35" s="5" t="n">
         <f aca="false">(C35+D35+E35)/3</f>
-        <v>0</v>
+        <v>240</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2177,19 +2197,19 @@
       </c>
       <c r="C36" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,1)</f>
-        <v>0</v>
+        <v>253</v>
       </c>
       <c r="D36" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,8)</f>
-        <v>0</v>
+        <v>305</v>
       </c>
       <c r="E36" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,10)</f>
-        <v>0</v>
+        <v>637</v>
       </c>
       <c r="F36" s="5" t="n">
         <f aca="false">(C36+D36+E36)/3</f>
-        <v>0</v>
+        <v>398.333333333333</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2202,19 +2222,19 @@
       </c>
       <c r="C37" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,1)</f>
-        <v>0</v>
+        <v>253</v>
       </c>
       <c r="D37" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,9)</f>
-        <v>0</v>
+        <v>162</v>
       </c>
       <c r="E37" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,10)</f>
-        <v>0</v>
+        <v>637</v>
       </c>
       <c r="F37" s="5" t="n">
         <f aca="false">(C37+D37+E37)/3</f>
-        <v>0</v>
+        <v>350.666666666667</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2227,19 +2247,19 @@
       </c>
       <c r="C38" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,2)</f>
-        <v>0</v>
+        <v>447</v>
       </c>
       <c r="D38" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,3)</f>
-        <v>0</v>
+        <v>669</v>
       </c>
       <c r="E38" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,4)</f>
-        <v>0</v>
+        <v>278</v>
       </c>
       <c r="F38" s="5" t="n">
         <f aca="false">(C38+D38+E38)/3</f>
-        <v>0</v>
+        <v>464.666666666667</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2252,19 +2272,19 @@
       </c>
       <c r="C39" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,2)</f>
-        <v>0</v>
+        <v>447</v>
       </c>
       <c r="D39" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,3)</f>
-        <v>0</v>
+        <v>669</v>
       </c>
       <c r="E39" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,5)</f>
-        <v>0</v>
+        <v>53</v>
       </c>
       <c r="F39" s="5" t="n">
         <f aca="false">(C39+D39+E39)/3</f>
-        <v>0</v>
+        <v>389.666666666667</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2277,19 +2297,19 @@
       </c>
       <c r="C40" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,2)</f>
-        <v>0</v>
+        <v>447</v>
       </c>
       <c r="D40" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,3)</f>
-        <v>0</v>
+        <v>669</v>
       </c>
       <c r="E40" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,6)</f>
-        <v>0</v>
+        <v>260</v>
       </c>
       <c r="F40" s="5" t="n">
         <f aca="false">(C40+D40+E40)/3</f>
-        <v>0</v>
+        <v>458.666666666667</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2302,19 +2322,19 @@
       </c>
       <c r="C41" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,2)</f>
-        <v>0</v>
+        <v>447</v>
       </c>
       <c r="D41" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,3)</f>
-        <v>0</v>
+        <v>669</v>
       </c>
       <c r="E41" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,7)</f>
-        <v>0</v>
+        <v>250</v>
       </c>
       <c r="F41" s="5" t="n">
         <f aca="false">(C41+D41+E41)/3</f>
-        <v>0</v>
+        <v>455.333333333333</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2327,19 +2347,19 @@
       </c>
       <c r="C42" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,2)</f>
-        <v>0</v>
+        <v>447</v>
       </c>
       <c r="D42" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,3)</f>
-        <v>0</v>
+        <v>669</v>
       </c>
       <c r="E42" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,8)</f>
-        <v>0</v>
+        <v>305</v>
       </c>
       <c r="F42" s="5" t="n">
         <f aca="false">(C42+D42+E42)/3</f>
-        <v>0</v>
+        <v>473.666666666667</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2352,19 +2372,19 @@
       </c>
       <c r="C43" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,2)</f>
-        <v>0</v>
+        <v>447</v>
       </c>
       <c r="D43" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,3)</f>
-        <v>0</v>
+        <v>669</v>
       </c>
       <c r="E43" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,9)</f>
-        <v>0</v>
+        <v>162</v>
       </c>
       <c r="F43" s="5" t="n">
         <f aca="false">(C43+D43+E43)/3</f>
-        <v>0</v>
+        <v>426</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2377,19 +2397,19 @@
       </c>
       <c r="C44" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,2)</f>
-        <v>0</v>
+        <v>447</v>
       </c>
       <c r="D44" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,3)</f>
-        <v>0</v>
+        <v>669</v>
       </c>
       <c r="E44" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,10)</f>
-        <v>0</v>
+        <v>637</v>
       </c>
       <c r="F44" s="5" t="n">
         <f aca="false">(C44+D44+E44)/3</f>
-        <v>0</v>
+        <v>584.333333333333</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2402,19 +2422,19 @@
       </c>
       <c r="C45" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,2)</f>
-        <v>0</v>
+        <v>447</v>
       </c>
       <c r="D45" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,4)</f>
-        <v>0</v>
+        <v>278</v>
       </c>
       <c r="E45" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,5)</f>
-        <v>0</v>
+        <v>53</v>
       </c>
       <c r="F45" s="5" t="n">
         <f aca="false">(C45+D45+E45)/3</f>
-        <v>0</v>
+        <v>259.333333333333</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2427,19 +2447,19 @@
       </c>
       <c r="C46" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,2)</f>
-        <v>0</v>
+        <v>447</v>
       </c>
       <c r="D46" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,4)</f>
-        <v>0</v>
+        <v>278</v>
       </c>
       <c r="E46" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,6)</f>
-        <v>0</v>
+        <v>260</v>
       </c>
       <c r="F46" s="5" t="n">
         <f aca="false">(C46+D46+E46)/3</f>
-        <v>0</v>
+        <v>328.333333333333</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2452,19 +2472,19 @@
       </c>
       <c r="C47" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,2)</f>
-        <v>0</v>
+        <v>447</v>
       </c>
       <c r="D47" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,4)</f>
-        <v>0</v>
+        <v>278</v>
       </c>
       <c r="E47" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,7)</f>
-        <v>0</v>
+        <v>250</v>
       </c>
       <c r="F47" s="5" t="n">
         <f aca="false">(C47+D47+E47)/3</f>
-        <v>0</v>
+        <v>325</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2477,19 +2497,19 @@
       </c>
       <c r="C48" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,2)</f>
-        <v>0</v>
+        <v>447</v>
       </c>
       <c r="D48" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,4)</f>
-        <v>0</v>
+        <v>278</v>
       </c>
       <c r="E48" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,8)</f>
-        <v>0</v>
+        <v>305</v>
       </c>
       <c r="F48" s="5" t="n">
         <f aca="false">(C48+D48+E48)/3</f>
-        <v>0</v>
+        <v>343.333333333333</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2502,19 +2522,19 @@
       </c>
       <c r="C49" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,2)</f>
-        <v>0</v>
+        <v>447</v>
       </c>
       <c r="D49" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,4)</f>
-        <v>0</v>
+        <v>278</v>
       </c>
       <c r="E49" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,9)</f>
-        <v>0</v>
+        <v>162</v>
       </c>
       <c r="F49" s="5" t="n">
         <f aca="false">(C49+D49+E49)/3</f>
-        <v>0</v>
+        <v>295.666666666667</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2527,19 +2547,19 @@
       </c>
       <c r="C50" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,2)</f>
-        <v>0</v>
+        <v>447</v>
       </c>
       <c r="D50" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,4)</f>
-        <v>0</v>
+        <v>278</v>
       </c>
       <c r="E50" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,10)</f>
-        <v>0</v>
+        <v>637</v>
       </c>
       <c r="F50" s="5" t="n">
         <f aca="false">(C50+D50+E50)/3</f>
-        <v>0</v>
+        <v>454</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2552,19 +2572,19 @@
       </c>
       <c r="C51" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,2)</f>
-        <v>0</v>
+        <v>447</v>
       </c>
       <c r="D51" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,5)</f>
-        <v>0</v>
+        <v>53</v>
       </c>
       <c r="E51" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,6)</f>
-        <v>0</v>
+        <v>260</v>
       </c>
       <c r="F51" s="5" t="n">
         <f aca="false">(C51+D51+E51)/3</f>
-        <v>0</v>
+        <v>253.333333333333</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2577,19 +2597,19 @@
       </c>
       <c r="C52" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,2)</f>
-        <v>0</v>
+        <v>447</v>
       </c>
       <c r="D52" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,5)</f>
-        <v>0</v>
+        <v>53</v>
       </c>
       <c r="E52" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,7)</f>
-        <v>0</v>
+        <v>250</v>
       </c>
       <c r="F52" s="5" t="n">
         <f aca="false">(C52+D52+E52)/3</f>
-        <v>0</v>
+        <v>250</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2602,19 +2622,19 @@
       </c>
       <c r="C53" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,2)</f>
-        <v>0</v>
+        <v>447</v>
       </c>
       <c r="D53" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,5)</f>
-        <v>0</v>
+        <v>53</v>
       </c>
       <c r="E53" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,8)</f>
-        <v>0</v>
+        <v>305</v>
       </c>
       <c r="F53" s="5" t="n">
         <f aca="false">(C53+D53+E53)/3</f>
-        <v>0</v>
+        <v>268.333333333333</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2627,19 +2647,19 @@
       </c>
       <c r="C54" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,2)</f>
-        <v>0</v>
+        <v>447</v>
       </c>
       <c r="D54" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,5)</f>
-        <v>0</v>
+        <v>53</v>
       </c>
       <c r="E54" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,9)</f>
-        <v>0</v>
+        <v>162</v>
       </c>
       <c r="F54" s="5" t="n">
         <f aca="false">(C54+D54+E54)/3</f>
-        <v>0</v>
+        <v>220.666666666667</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2652,19 +2672,19 @@
       </c>
       <c r="C55" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,2)</f>
-        <v>0</v>
+        <v>447</v>
       </c>
       <c r="D55" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,5)</f>
-        <v>0</v>
+        <v>53</v>
       </c>
       <c r="E55" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,10)</f>
-        <v>0</v>
+        <v>637</v>
       </c>
       <c r="F55" s="5" t="n">
         <f aca="false">(C55+D55+E55)/3</f>
-        <v>0</v>
+        <v>379</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2677,19 +2697,19 @@
       </c>
       <c r="C56" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,2)</f>
-        <v>0</v>
+        <v>447</v>
       </c>
       <c r="D56" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,6)</f>
-        <v>0</v>
+        <v>260</v>
       </c>
       <c r="E56" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,7)</f>
-        <v>0</v>
+        <v>250</v>
       </c>
       <c r="F56" s="5" t="n">
         <f aca="false">(C56+D56+E56)/3</f>
-        <v>0</v>
+        <v>319</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2702,19 +2722,19 @@
       </c>
       <c r="C57" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,2)</f>
-        <v>0</v>
+        <v>447</v>
       </c>
       <c r="D57" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,6)</f>
-        <v>0</v>
+        <v>260</v>
       </c>
       <c r="E57" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,8)</f>
-        <v>0</v>
+        <v>305</v>
       </c>
       <c r="F57" s="5" t="n">
         <f aca="false">(C57+D57+E57)/3</f>
-        <v>0</v>
+        <v>337.333333333333</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2727,19 +2747,19 @@
       </c>
       <c r="C58" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,2)</f>
-        <v>0</v>
+        <v>447</v>
       </c>
       <c r="D58" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,6)</f>
-        <v>0</v>
+        <v>260</v>
       </c>
       <c r="E58" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,9)</f>
-        <v>0</v>
+        <v>162</v>
       </c>
       <c r="F58" s="5" t="n">
         <f aca="false">(C58+D58+E58)/3</f>
-        <v>0</v>
+        <v>289.666666666667</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2752,19 +2772,19 @@
       </c>
       <c r="C59" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,2)</f>
-        <v>0</v>
+        <v>447</v>
       </c>
       <c r="D59" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,6)</f>
-        <v>0</v>
+        <v>260</v>
       </c>
       <c r="E59" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,10)</f>
-        <v>0</v>
+        <v>637</v>
       </c>
       <c r="F59" s="5" t="n">
         <f aca="false">(C59+D59+E59)/3</f>
-        <v>0</v>
+        <v>448</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2777,19 +2797,19 @@
       </c>
       <c r="C60" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,2)</f>
-        <v>0</v>
+        <v>447</v>
       </c>
       <c r="D60" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,7)</f>
-        <v>0</v>
+        <v>250</v>
       </c>
       <c r="E60" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,8)</f>
-        <v>0</v>
+        <v>305</v>
       </c>
       <c r="F60" s="5" t="n">
         <f aca="false">(C60+D60+E60)/3</f>
-        <v>0</v>
+        <v>334</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2802,19 +2822,19 @@
       </c>
       <c r="C61" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,2)</f>
-        <v>0</v>
+        <v>447</v>
       </c>
       <c r="D61" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,7)</f>
-        <v>0</v>
+        <v>250</v>
       </c>
       <c r="E61" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,9)</f>
-        <v>0</v>
+        <v>162</v>
       </c>
       <c r="F61" s="5" t="n">
         <f aca="false">(C61+D61+E61)/3</f>
-        <v>0</v>
+        <v>286.333333333333</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2827,19 +2847,19 @@
       </c>
       <c r="C62" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,2)</f>
-        <v>0</v>
+        <v>447</v>
       </c>
       <c r="D62" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,7)</f>
-        <v>0</v>
+        <v>250</v>
       </c>
       <c r="E62" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,10)</f>
-        <v>0</v>
+        <v>637</v>
       </c>
       <c r="F62" s="5" t="n">
         <f aca="false">(C62+D62+E62)/3</f>
-        <v>0</v>
+        <v>444.666666666667</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2852,19 +2872,19 @@
       </c>
       <c r="C63" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,2)</f>
-        <v>0</v>
+        <v>447</v>
       </c>
       <c r="D63" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,8)</f>
-        <v>0</v>
+        <v>305</v>
       </c>
       <c r="E63" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,9)</f>
-        <v>0</v>
+        <v>162</v>
       </c>
       <c r="F63" s="5" t="n">
         <f aca="false">(C63+D63+E63)/3</f>
-        <v>0</v>
+        <v>304.666666666667</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2877,19 +2897,19 @@
       </c>
       <c r="C64" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,2)</f>
-        <v>0</v>
+        <v>447</v>
       </c>
       <c r="D64" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,8)</f>
-        <v>0</v>
+        <v>305</v>
       </c>
       <c r="E64" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,10)</f>
-        <v>0</v>
+        <v>637</v>
       </c>
       <c r="F64" s="5" t="n">
         <f aca="false">(C64+D64+E64)/3</f>
-        <v>0</v>
+        <v>463</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2902,19 +2922,19 @@
       </c>
       <c r="C65" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,2)</f>
-        <v>0</v>
+        <v>447</v>
       </c>
       <c r="D65" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,9)</f>
-        <v>0</v>
+        <v>162</v>
       </c>
       <c r="E65" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,10)</f>
-        <v>0</v>
+        <v>637</v>
       </c>
       <c r="F65" s="5" t="n">
         <f aca="false">(C65+D65+E65)/3</f>
-        <v>0</v>
+        <v>415.333333333333</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2927,19 +2947,19 @@
       </c>
       <c r="C66" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,3)</f>
-        <v>0</v>
+        <v>669</v>
       </c>
       <c r="D66" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,4)</f>
-        <v>0</v>
+        <v>278</v>
       </c>
       <c r="E66" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,5)</f>
-        <v>0</v>
+        <v>53</v>
       </c>
       <c r="F66" s="5" t="n">
         <f aca="false">(C66+D66+E66)/3</f>
-        <v>0</v>
+        <v>333.333333333333</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2952,19 +2972,19 @@
       </c>
       <c r="C67" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,3)</f>
-        <v>0</v>
+        <v>669</v>
       </c>
       <c r="D67" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,4)</f>
-        <v>0</v>
+        <v>278</v>
       </c>
       <c r="E67" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,6)</f>
-        <v>0</v>
+        <v>260</v>
       </c>
       <c r="F67" s="5" t="n">
         <f aca="false">(C67+D67+E67)/3</f>
-        <v>0</v>
+        <v>402.333333333333</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2977,19 +2997,19 @@
       </c>
       <c r="C68" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,3)</f>
-        <v>0</v>
+        <v>669</v>
       </c>
       <c r="D68" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,4)</f>
-        <v>0</v>
+        <v>278</v>
       </c>
       <c r="E68" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,7)</f>
-        <v>0</v>
+        <v>250</v>
       </c>
       <c r="F68" s="5" t="n">
         <f aca="false">(C68+D68+E68)/3</f>
-        <v>0</v>
+        <v>399</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3002,19 +3022,19 @@
       </c>
       <c r="C69" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,3)</f>
-        <v>0</v>
+        <v>669</v>
       </c>
       <c r="D69" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,4)</f>
-        <v>0</v>
+        <v>278</v>
       </c>
       <c r="E69" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,8)</f>
-        <v>0</v>
+        <v>305</v>
       </c>
       <c r="F69" s="5" t="n">
         <f aca="false">(C69+D69+E69)/3</f>
-        <v>0</v>
+        <v>417.333333333333</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3027,19 +3047,19 @@
       </c>
       <c r="C70" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,3)</f>
-        <v>0</v>
+        <v>669</v>
       </c>
       <c r="D70" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,4)</f>
-        <v>0</v>
+        <v>278</v>
       </c>
       <c r="E70" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,9)</f>
-        <v>0</v>
+        <v>162</v>
       </c>
       <c r="F70" s="5" t="n">
         <f aca="false">(C70+D70+E70)/3</f>
-        <v>0</v>
+        <v>369.666666666667</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3052,19 +3072,19 @@
       </c>
       <c r="C71" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,3)</f>
-        <v>0</v>
+        <v>669</v>
       </c>
       <c r="D71" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,4)</f>
-        <v>0</v>
+        <v>278</v>
       </c>
       <c r="E71" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,10)</f>
-        <v>0</v>
+        <v>637</v>
       </c>
       <c r="F71" s="5" t="n">
         <f aca="false">(C71+D71+E71)/3</f>
-        <v>0</v>
+        <v>528</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3077,19 +3097,19 @@
       </c>
       <c r="C72" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,3)</f>
-        <v>0</v>
+        <v>669</v>
       </c>
       <c r="D72" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,5)</f>
-        <v>0</v>
+        <v>53</v>
       </c>
       <c r="E72" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,6)</f>
-        <v>0</v>
+        <v>260</v>
       </c>
       <c r="F72" s="5" t="n">
         <f aca="false">(C72+D72+E72)/3</f>
-        <v>0</v>
+        <v>327.333333333333</v>
       </c>
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3102,19 +3122,19 @@
       </c>
       <c r="C73" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,3)</f>
-        <v>0</v>
+        <v>669</v>
       </c>
       <c r="D73" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,5)</f>
-        <v>0</v>
+        <v>53</v>
       </c>
       <c r="E73" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,7)</f>
-        <v>0</v>
+        <v>250</v>
       </c>
       <c r="F73" s="5" t="n">
         <f aca="false">(C73+D73+E73)/3</f>
-        <v>0</v>
+        <v>324</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3127,19 +3147,19 @@
       </c>
       <c r="C74" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,3)</f>
-        <v>0</v>
+        <v>669</v>
       </c>
       <c r="D74" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,5)</f>
-        <v>0</v>
+        <v>53</v>
       </c>
       <c r="E74" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,8)</f>
-        <v>0</v>
+        <v>305</v>
       </c>
       <c r="F74" s="5" t="n">
         <f aca="false">(C74+D74+E74)/3</f>
-        <v>0</v>
+        <v>342.333333333333</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3152,19 +3172,19 @@
       </c>
       <c r="C75" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,3)</f>
-        <v>0</v>
+        <v>669</v>
       </c>
       <c r="D75" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,5)</f>
-        <v>0</v>
+        <v>53</v>
       </c>
       <c r="E75" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,9)</f>
-        <v>0</v>
+        <v>162</v>
       </c>
       <c r="F75" s="5" t="n">
         <f aca="false">(C75+D75+E75)/3</f>
-        <v>0</v>
+        <v>294.666666666667</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3177,19 +3197,19 @@
       </c>
       <c r="C76" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,3)</f>
-        <v>0</v>
+        <v>669</v>
       </c>
       <c r="D76" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,5)</f>
-        <v>0</v>
+        <v>53</v>
       </c>
       <c r="E76" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,10)</f>
-        <v>0</v>
+        <v>637</v>
       </c>
       <c r="F76" s="5" t="n">
         <f aca="false">(C76+D76+E76)/3</f>
-        <v>0</v>
+        <v>453</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3202,19 +3222,19 @@
       </c>
       <c r="C77" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,3)</f>
-        <v>0</v>
+        <v>669</v>
       </c>
       <c r="D77" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,6)</f>
-        <v>0</v>
+        <v>260</v>
       </c>
       <c r="E77" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,7)</f>
-        <v>0</v>
+        <v>250</v>
       </c>
       <c r="F77" s="5" t="n">
         <f aca="false">(C77+D77+E77)/3</f>
-        <v>0</v>
+        <v>393</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3227,19 +3247,19 @@
       </c>
       <c r="C78" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,3)</f>
-        <v>0</v>
+        <v>669</v>
       </c>
       <c r="D78" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,6)</f>
-        <v>0</v>
+        <v>260</v>
       </c>
       <c r="E78" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,8)</f>
-        <v>0</v>
+        <v>305</v>
       </c>
       <c r="F78" s="5" t="n">
         <f aca="false">(C78+D78+E78)/3</f>
-        <v>0</v>
+        <v>411.333333333333</v>
       </c>
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3252,19 +3272,19 @@
       </c>
       <c r="C79" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,3)</f>
-        <v>0</v>
+        <v>669</v>
       </c>
       <c r="D79" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,6)</f>
-        <v>0</v>
+        <v>260</v>
       </c>
       <c r="E79" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,9)</f>
-        <v>0</v>
+        <v>162</v>
       </c>
       <c r="F79" s="5" t="n">
         <f aca="false">(C79+D79+E79)/3</f>
-        <v>0</v>
+        <v>363.666666666667</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3277,19 +3297,19 @@
       </c>
       <c r="C80" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,3)</f>
-        <v>0</v>
+        <v>669</v>
       </c>
       <c r="D80" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,6)</f>
-        <v>0</v>
+        <v>260</v>
       </c>
       <c r="E80" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,10)</f>
-        <v>0</v>
+        <v>637</v>
       </c>
       <c r="F80" s="5" t="n">
         <f aca="false">(C80+D80+E80)/3</f>
-        <v>0</v>
+        <v>522</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3302,19 +3322,19 @@
       </c>
       <c r="C81" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,3)</f>
-        <v>0</v>
+        <v>669</v>
       </c>
       <c r="D81" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,7)</f>
-        <v>0</v>
+        <v>250</v>
       </c>
       <c r="E81" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,8)</f>
-        <v>0</v>
+        <v>305</v>
       </c>
       <c r="F81" s="5" t="n">
         <f aca="false">(C81+D81+E81)/3</f>
-        <v>0</v>
+        <v>408</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3327,19 +3347,19 @@
       </c>
       <c r="C82" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,3)</f>
-        <v>0</v>
+        <v>669</v>
       </c>
       <c r="D82" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,7)</f>
-        <v>0</v>
+        <v>250</v>
       </c>
       <c r="E82" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,9)</f>
-        <v>0</v>
+        <v>162</v>
       </c>
       <c r="F82" s="5" t="n">
         <f aca="false">(C82+D82+E82)/3</f>
-        <v>0</v>
+        <v>360.333333333333</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3352,19 +3372,19 @@
       </c>
       <c r="C83" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,3)</f>
-        <v>0</v>
+        <v>669</v>
       </c>
       <c r="D83" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,7)</f>
-        <v>0</v>
+        <v>250</v>
       </c>
       <c r="E83" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,10)</f>
-        <v>0</v>
+        <v>637</v>
       </c>
       <c r="F83" s="5" t="n">
         <f aca="false">(C83+D83+E83)/3</f>
-        <v>0</v>
+        <v>518.666666666667</v>
       </c>
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3377,19 +3397,19 @@
       </c>
       <c r="C84" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,3)</f>
-        <v>0</v>
+        <v>669</v>
       </c>
       <c r="D84" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,8)</f>
-        <v>0</v>
+        <v>305</v>
       </c>
       <c r="E84" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,9)</f>
-        <v>0</v>
+        <v>162</v>
       </c>
       <c r="F84" s="5" t="n">
         <f aca="false">(C84+D84+E84)/3</f>
-        <v>0</v>
+        <v>378.666666666667</v>
       </c>
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3402,19 +3422,19 @@
       </c>
       <c r="C85" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,3)</f>
-        <v>0</v>
+        <v>669</v>
       </c>
       <c r="D85" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,8)</f>
-        <v>0</v>
+        <v>305</v>
       </c>
       <c r="E85" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,10)</f>
-        <v>0</v>
+        <v>637</v>
       </c>
       <c r="F85" s="5" t="n">
         <f aca="false">(C85+D85+E85)/3</f>
-        <v>0</v>
+        <v>537</v>
       </c>
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3427,19 +3447,19 @@
       </c>
       <c r="C86" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,3)</f>
-        <v>0</v>
+        <v>669</v>
       </c>
       <c r="D86" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,9)</f>
-        <v>0</v>
+        <v>162</v>
       </c>
       <c r="E86" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,10)</f>
-        <v>0</v>
+        <v>637</v>
       </c>
       <c r="F86" s="5" t="n">
         <f aca="false">(C86+D86+E86)/3</f>
-        <v>0</v>
+        <v>489.333333333333</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3452,19 +3472,19 @@
       </c>
       <c r="C87" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,4)</f>
-        <v>0</v>
+        <v>278</v>
       </c>
       <c r="D87" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,5)</f>
-        <v>0</v>
+        <v>53</v>
       </c>
       <c r="E87" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,6)</f>
-        <v>0</v>
+        <v>260</v>
       </c>
       <c r="F87" s="5" t="n">
         <f aca="false">(C87+D87+E87)/3</f>
-        <v>0</v>
+        <v>197</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3477,19 +3497,19 @@
       </c>
       <c r="C88" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,4)</f>
-        <v>0</v>
+        <v>278</v>
       </c>
       <c r="D88" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,5)</f>
-        <v>0</v>
+        <v>53</v>
       </c>
       <c r="E88" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,7)</f>
-        <v>0</v>
+        <v>250</v>
       </c>
       <c r="F88" s="5" t="n">
         <f aca="false">(C88+D88+E88)/3</f>
-        <v>0</v>
+        <v>193.666666666667</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3502,19 +3522,19 @@
       </c>
       <c r="C89" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,4)</f>
-        <v>0</v>
+        <v>278</v>
       </c>
       <c r="D89" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,5)</f>
-        <v>0</v>
+        <v>53</v>
       </c>
       <c r="E89" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,8)</f>
-        <v>0</v>
+        <v>305</v>
       </c>
       <c r="F89" s="5" t="n">
         <f aca="false">(C89+D89+E89)/3</f>
-        <v>0</v>
+        <v>212</v>
       </c>
     </row>
     <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3527,19 +3547,19 @@
       </c>
       <c r="C90" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,4)</f>
-        <v>0</v>
+        <v>278</v>
       </c>
       <c r="D90" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,5)</f>
-        <v>0</v>
+        <v>53</v>
       </c>
       <c r="E90" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,9)</f>
-        <v>0</v>
+        <v>162</v>
       </c>
       <c r="F90" s="5" t="n">
         <f aca="false">(C90+D90+E90)/3</f>
-        <v>0</v>
+        <v>164.333333333333</v>
       </c>
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3552,19 +3572,19 @@
       </c>
       <c r="C91" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,4)</f>
-        <v>0</v>
+        <v>278</v>
       </c>
       <c r="D91" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,5)</f>
-        <v>0</v>
+        <v>53</v>
       </c>
       <c r="E91" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,10)</f>
-        <v>0</v>
+        <v>637</v>
       </c>
       <c r="F91" s="5" t="n">
         <f aca="false">(C91+D91+E91)/3</f>
-        <v>0</v>
+        <v>322.666666666667</v>
       </c>
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3577,19 +3597,19 @@
       </c>
       <c r="C92" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,4)</f>
-        <v>0</v>
+        <v>278</v>
       </c>
       <c r="D92" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,6)</f>
-        <v>0</v>
+        <v>260</v>
       </c>
       <c r="E92" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,7)</f>
-        <v>0</v>
+        <v>250</v>
       </c>
       <c r="F92" s="5" t="n">
         <f aca="false">(C92+D92+E92)/3</f>
-        <v>0</v>
+        <v>262.666666666667</v>
       </c>
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3602,19 +3622,19 @@
       </c>
       <c r="C93" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,4)</f>
-        <v>0</v>
+        <v>278</v>
       </c>
       <c r="D93" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,6)</f>
-        <v>0</v>
+        <v>260</v>
       </c>
       <c r="E93" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,8)</f>
-        <v>0</v>
+        <v>305</v>
       </c>
       <c r="F93" s="5" t="n">
         <f aca="false">(C93+D93+E93)/3</f>
-        <v>0</v>
+        <v>281</v>
       </c>
     </row>
     <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3627,19 +3647,19 @@
       </c>
       <c r="C94" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,4)</f>
-        <v>0</v>
+        <v>278</v>
       </c>
       <c r="D94" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,6)</f>
-        <v>0</v>
+        <v>260</v>
       </c>
       <c r="E94" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,9)</f>
-        <v>0</v>
+        <v>162</v>
       </c>
       <c r="F94" s="5" t="n">
         <f aca="false">(C94+D94+E94)/3</f>
-        <v>0</v>
+        <v>233.333333333333</v>
       </c>
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3652,19 +3672,19 @@
       </c>
       <c r="C95" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,4)</f>
-        <v>0</v>
+        <v>278</v>
       </c>
       <c r="D95" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,6)</f>
-        <v>0</v>
+        <v>260</v>
       </c>
       <c r="E95" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,10)</f>
-        <v>0</v>
+        <v>637</v>
       </c>
       <c r="F95" s="5" t="n">
         <f aca="false">(C95+D95+E95)/3</f>
-        <v>0</v>
+        <v>391.666666666667</v>
       </c>
     </row>
     <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3677,19 +3697,19 @@
       </c>
       <c r="C96" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,4)</f>
-        <v>0</v>
+        <v>278</v>
       </c>
       <c r="D96" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,7)</f>
-        <v>0</v>
+        <v>250</v>
       </c>
       <c r="E96" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,8)</f>
-        <v>0</v>
+        <v>305</v>
       </c>
       <c r="F96" s="5" t="n">
         <f aca="false">(C96+D96+E96)/3</f>
-        <v>0</v>
+        <v>277.666666666667</v>
       </c>
     </row>
     <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3702,19 +3722,19 @@
       </c>
       <c r="C97" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,4)</f>
-        <v>0</v>
+        <v>278</v>
       </c>
       <c r="D97" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,7)</f>
-        <v>0</v>
+        <v>250</v>
       </c>
       <c r="E97" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,9)</f>
-        <v>0</v>
+        <v>162</v>
       </c>
       <c r="F97" s="5" t="n">
         <f aca="false">(C97+D97+E97)/3</f>
-        <v>0</v>
+        <v>230</v>
       </c>
     </row>
     <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3727,19 +3747,19 @@
       </c>
       <c r="C98" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,4)</f>
-        <v>0</v>
+        <v>278</v>
       </c>
       <c r="D98" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,7)</f>
-        <v>0</v>
+        <v>250</v>
       </c>
       <c r="E98" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,10)</f>
-        <v>0</v>
+        <v>637</v>
       </c>
       <c r="F98" s="5" t="n">
         <f aca="false">(C98+D98+E98)/3</f>
-        <v>0</v>
+        <v>388.333333333333</v>
       </c>
     </row>
     <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3752,19 +3772,19 @@
       </c>
       <c r="C99" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,4)</f>
-        <v>0</v>
+        <v>278</v>
       </c>
       <c r="D99" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,8)</f>
-        <v>0</v>
+        <v>305</v>
       </c>
       <c r="E99" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,9)</f>
-        <v>0</v>
+        <v>162</v>
       </c>
       <c r="F99" s="5" t="n">
         <f aca="false">(C99+D99+E99)/3</f>
-        <v>0</v>
+        <v>248.333333333333</v>
       </c>
     </row>
     <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3777,19 +3797,19 @@
       </c>
       <c r="C100" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,4)</f>
-        <v>0</v>
+        <v>278</v>
       </c>
       <c r="D100" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,8)</f>
-        <v>0</v>
+        <v>305</v>
       </c>
       <c r="E100" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,10)</f>
-        <v>0</v>
+        <v>637</v>
       </c>
       <c r="F100" s="5" t="n">
         <f aca="false">(C100+D100+E100)/3</f>
-        <v>0</v>
+        <v>406.666666666667</v>
       </c>
     </row>
     <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3802,19 +3822,19 @@
       </c>
       <c r="C101" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,4)</f>
-        <v>0</v>
+        <v>278</v>
       </c>
       <c r="D101" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,9)</f>
-        <v>0</v>
+        <v>162</v>
       </c>
       <c r="E101" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,10)</f>
-        <v>0</v>
+        <v>637</v>
       </c>
       <c r="F101" s="5" t="n">
         <f aca="false">(C101+D101+E101)/3</f>
-        <v>0</v>
+        <v>359</v>
       </c>
     </row>
     <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3827,19 +3847,19 @@
       </c>
       <c r="C102" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,5)</f>
-        <v>0</v>
+        <v>53</v>
       </c>
       <c r="D102" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,6)</f>
-        <v>0</v>
+        <v>260</v>
       </c>
       <c r="E102" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,7)</f>
-        <v>0</v>
+        <v>250</v>
       </c>
       <c r="F102" s="5" t="n">
         <f aca="false">(C102+D102+E102)/3</f>
-        <v>0</v>
+        <v>187.666666666667</v>
       </c>
     </row>
     <row r="103" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3852,19 +3872,19 @@
       </c>
       <c r="C103" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,5)</f>
-        <v>0</v>
+        <v>53</v>
       </c>
       <c r="D103" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,6)</f>
-        <v>0</v>
+        <v>260</v>
       </c>
       <c r="E103" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,8)</f>
-        <v>0</v>
+        <v>305</v>
       </c>
       <c r="F103" s="5" t="n">
         <f aca="false">(C103+D103+E103)/3</f>
-        <v>0</v>
+        <v>206</v>
       </c>
     </row>
     <row r="104" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3877,19 +3897,19 @@
       </c>
       <c r="C104" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,5)</f>
-        <v>0</v>
+        <v>53</v>
       </c>
       <c r="D104" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,6)</f>
-        <v>0</v>
+        <v>260</v>
       </c>
       <c r="E104" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,9)</f>
-        <v>0</v>
+        <v>162</v>
       </c>
       <c r="F104" s="5" t="n">
         <f aca="false">(C104+D104+E104)/3</f>
-        <v>0</v>
+        <v>158.333333333333</v>
       </c>
     </row>
     <row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3902,19 +3922,19 @@
       </c>
       <c r="C105" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,5)</f>
-        <v>0</v>
+        <v>53</v>
       </c>
       <c r="D105" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,6)</f>
-        <v>0</v>
+        <v>260</v>
       </c>
       <c r="E105" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,10)</f>
-        <v>0</v>
+        <v>637</v>
       </c>
       <c r="F105" s="5" t="n">
         <f aca="false">(C105+D105+E105)/3</f>
-        <v>0</v>
+        <v>316.666666666667</v>
       </c>
     </row>
     <row r="106" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3927,19 +3947,19 @@
       </c>
       <c r="C106" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,5)</f>
-        <v>0</v>
+        <v>53</v>
       </c>
       <c r="D106" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,7)</f>
-        <v>0</v>
+        <v>250</v>
       </c>
       <c r="E106" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,8)</f>
-        <v>0</v>
+        <v>305</v>
       </c>
       <c r="F106" s="5" t="n">
         <f aca="false">(C106+D106+E106)/3</f>
-        <v>0</v>
+        <v>202.666666666667</v>
       </c>
     </row>
     <row r="107" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3952,19 +3972,19 @@
       </c>
       <c r="C107" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,5)</f>
-        <v>0</v>
+        <v>53</v>
       </c>
       <c r="D107" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,7)</f>
-        <v>0</v>
+        <v>250</v>
       </c>
       <c r="E107" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,9)</f>
-        <v>0</v>
+        <v>162</v>
       </c>
       <c r="F107" s="5" t="n">
         <f aca="false">(C107+D107+E107)/3</f>
-        <v>0</v>
+        <v>155</v>
       </c>
     </row>
     <row r="108" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3977,19 +3997,19 @@
       </c>
       <c r="C108" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,5)</f>
-        <v>0</v>
+        <v>53</v>
       </c>
       <c r="D108" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,7)</f>
-        <v>0</v>
+        <v>250</v>
       </c>
       <c r="E108" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,10)</f>
-        <v>0</v>
+        <v>637</v>
       </c>
       <c r="F108" s="5" t="n">
         <f aca="false">(C108+D108+E108)/3</f>
-        <v>0</v>
+        <v>313.333333333333</v>
       </c>
     </row>
     <row r="109" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4002,19 +4022,19 @@
       </c>
       <c r="C109" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,5)</f>
-        <v>0</v>
+        <v>53</v>
       </c>
       <c r="D109" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,8)</f>
-        <v>0</v>
+        <v>305</v>
       </c>
       <c r="E109" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,9)</f>
-        <v>0</v>
+        <v>162</v>
       </c>
       <c r="F109" s="5" t="n">
         <f aca="false">(C109+D109+E109)/3</f>
-        <v>0</v>
+        <v>173.333333333333</v>
       </c>
     </row>
     <row r="110" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4027,19 +4047,19 @@
       </c>
       <c r="C110" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,5)</f>
-        <v>0</v>
+        <v>53</v>
       </c>
       <c r="D110" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,8)</f>
-        <v>0</v>
+        <v>305</v>
       </c>
       <c r="E110" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,10)</f>
-        <v>0</v>
+        <v>637</v>
       </c>
       <c r="F110" s="5" t="n">
         <f aca="false">(C110+D110+E110)/3</f>
-        <v>0</v>
+        <v>331.666666666667</v>
       </c>
     </row>
     <row r="111" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4052,19 +4072,19 @@
       </c>
       <c r="C111" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,5)</f>
-        <v>0</v>
+        <v>53</v>
       </c>
       <c r="D111" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,9)</f>
-        <v>0</v>
+        <v>162</v>
       </c>
       <c r="E111" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,10)</f>
-        <v>0</v>
+        <v>637</v>
       </c>
       <c r="F111" s="5" t="n">
         <f aca="false">(C111+D111+E111)/3</f>
-        <v>0</v>
+        <v>284</v>
       </c>
     </row>
     <row r="112" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4077,19 +4097,19 @@
       </c>
       <c r="C112" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,6)</f>
-        <v>0</v>
+        <v>260</v>
       </c>
       <c r="D112" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,7)</f>
-        <v>0</v>
+        <v>250</v>
       </c>
       <c r="E112" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,8)</f>
-        <v>0</v>
+        <v>305</v>
       </c>
       <c r="F112" s="5" t="n">
         <f aca="false">(C112+D112+E112)/3</f>
-        <v>0</v>
+        <v>271.666666666667</v>
       </c>
     </row>
     <row r="113" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4102,19 +4122,19 @@
       </c>
       <c r="C113" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,6)</f>
-        <v>0</v>
+        <v>260</v>
       </c>
       <c r="D113" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,7)</f>
-        <v>0</v>
+        <v>250</v>
       </c>
       <c r="E113" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,9)</f>
-        <v>0</v>
+        <v>162</v>
       </c>
       <c r="F113" s="5" t="n">
         <f aca="false">(C113+D113+E113)/3</f>
-        <v>0</v>
+        <v>224</v>
       </c>
     </row>
     <row r="114" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4127,19 +4147,19 @@
       </c>
       <c r="C114" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,6)</f>
-        <v>0</v>
+        <v>260</v>
       </c>
       <c r="D114" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,7)</f>
-        <v>0</v>
+        <v>250</v>
       </c>
       <c r="E114" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,10)</f>
-        <v>0</v>
+        <v>637</v>
       </c>
       <c r="F114" s="5" t="n">
         <f aca="false">(C114+D114+E114)/3</f>
-        <v>0</v>
+        <v>382.333333333333</v>
       </c>
     </row>
     <row r="115" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4152,19 +4172,19 @@
       </c>
       <c r="C115" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,6)</f>
-        <v>0</v>
+        <v>260</v>
       </c>
       <c r="D115" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,8)</f>
-        <v>0</v>
+        <v>305</v>
       </c>
       <c r="E115" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,9)</f>
-        <v>0</v>
+        <v>162</v>
       </c>
       <c r="F115" s="5" t="n">
         <f aca="false">(C115+D115+E115)/3</f>
-        <v>0</v>
+        <v>242.333333333333</v>
       </c>
     </row>
     <row r="116" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4177,19 +4197,19 @@
       </c>
       <c r="C116" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,6)</f>
-        <v>0</v>
+        <v>260</v>
       </c>
       <c r="D116" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,8)</f>
-        <v>0</v>
+        <v>305</v>
       </c>
       <c r="E116" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,10)</f>
-        <v>0</v>
+        <v>637</v>
       </c>
       <c r="F116" s="5" t="n">
         <f aca="false">(C116+D116+E116)/3</f>
-        <v>0</v>
+        <v>400.666666666667</v>
       </c>
     </row>
     <row r="117" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4202,19 +4222,19 @@
       </c>
       <c r="C117" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,6)</f>
-        <v>0</v>
+        <v>260</v>
       </c>
       <c r="D117" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,9)</f>
-        <v>0</v>
+        <v>162</v>
       </c>
       <c r="E117" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,10)</f>
-        <v>0</v>
+        <v>637</v>
       </c>
       <c r="F117" s="5" t="n">
         <f aca="false">(C117+D117+E117)/3</f>
-        <v>0</v>
+        <v>353</v>
       </c>
     </row>
     <row r="118" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4227,19 +4247,19 @@
       </c>
       <c r="C118" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,7)</f>
-        <v>0</v>
+        <v>250</v>
       </c>
       <c r="D118" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,8)</f>
-        <v>0</v>
+        <v>305</v>
       </c>
       <c r="E118" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,9)</f>
-        <v>0</v>
+        <v>162</v>
       </c>
       <c r="F118" s="5" t="n">
         <f aca="false">(C118+D118+E118)/3</f>
-        <v>0</v>
+        <v>239</v>
       </c>
     </row>
     <row r="119" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4252,19 +4272,19 @@
       </c>
       <c r="C119" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,7)</f>
-        <v>0</v>
+        <v>250</v>
       </c>
       <c r="D119" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,8)</f>
-        <v>0</v>
+        <v>305</v>
       </c>
       <c r="E119" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,10)</f>
-        <v>0</v>
+        <v>637</v>
       </c>
       <c r="F119" s="5" t="n">
         <f aca="false">(C119+D119+E119)/3</f>
-        <v>0</v>
+        <v>397.333333333333</v>
       </c>
     </row>
     <row r="120" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4277,19 +4297,19 @@
       </c>
       <c r="C120" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,7)</f>
-        <v>0</v>
+        <v>250</v>
       </c>
       <c r="D120" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,9)</f>
-        <v>0</v>
+        <v>162</v>
       </c>
       <c r="E120" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,10)</f>
-        <v>0</v>
+        <v>637</v>
       </c>
       <c r="F120" s="5" t="n">
         <f aca="false">(C120+D120+E120)/3</f>
-        <v>0</v>
+        <v>349.666666666667</v>
       </c>
     </row>
     <row r="121" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4302,19 +4322,19 @@
       </c>
       <c r="C121" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,8)</f>
-        <v>0</v>
+        <v>305</v>
       </c>
       <c r="D121" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,9)</f>
-        <v>0</v>
+        <v>162</v>
       </c>
       <c r="E121" s="2" t="n">
         <f aca="false">INDEX(Задача2!$B$7:$K$7,10)</f>
-        <v>0</v>
+        <v>637</v>
       </c>
       <c r="F121" s="5" t="n">
         <f aca="false">(C121+D121+E121)/3</f>
-        <v>0</v>
+        <v>368</v>
       </c>
     </row>
   </sheetData>

</xml_diff>